<commit_message>
Update VabLab Analysis Plan Template.xlsx
</commit_message>
<xml_diff>
--- a/VabLab Analysis Plan Template.xlsx
+++ b/VabLab Analysis Plan Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jillyhebert/Documents/Projects/RDA Work/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jillyhebert/Documents/GitHub/Analysis-Plan-Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{367C1BE4-1D00-534E-8458-D36941169EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32912027-5FF4-5147-A629-8B5D8AA9A2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="72980" yWindow="-880" windowWidth="33600" windowHeight="20400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="72960" yWindow="-880" windowWidth="33600" windowHeight="20400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
   <si>
     <t>Topic</t>
   </si>
@@ -58,9 +58,6 @@
     <t>Background:</t>
   </si>
   <si>
-    <t>What is the motivation for this work (~3 stentences)</t>
-  </si>
-  <si>
     <t>What analyses currently exist that are related or similar to your plan? Did they motivate you to pursue this project? (Within or outside of your team; list publications, preprints, talks/posters; can be non-exhaustive)</t>
   </si>
   <si>
@@ -70,16 +67,7 @@
     <t>State data set and put a link to the website and codebook</t>
   </si>
   <si>
-    <t xml:space="preserve">Brief summary of the data (cross sectional; longitudinal). Any oversamples or specific benifits of this data source? Study period: did you subsets data being used? </t>
-  </si>
-  <si>
     <t xml:space="preserve">How can the data be accessed? Is the data publicly available or are you using restricted data as well? </t>
-  </si>
-  <si>
-    <t>Eligiblity criteria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Any exlcusions from the eligible to the analytic sample? </t>
   </si>
   <si>
     <t xml:space="preserve">How many analyses have you already done using this dataset? (can be approximate, e.g. &gt;10) </t>
@@ -138,9 +126,6 @@
     <t xml:space="preserve">Model specification (variables, interactions) </t>
   </si>
   <si>
-    <t>Modeling strengths (e.g. justificaiton for choosing this model)</t>
-  </si>
-  <si>
     <t>Modeling limitations (e.g. concerns about what primary modeling approach may miss)</t>
   </si>
   <si>
@@ -174,23 +159,6 @@
     <t>Lead analyst</t>
   </si>
   <si>
-    <t>Number of people in the analytic sample and number of obersations (if repeated outcome measures)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Implementation steps: Copy this analysis plan to your prefered enviornment. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>Fill out the initial analysis plan based on your project. Update the analysis plan as decisions are made; that is, whenever you make updates to the analysis or change coding choices, you should have this document open to record changes to the planned analysis. Remeber this plan is to help promote reproducible reserach and will eventually be posted online. This document is for you, so modify it however you see fit!</t>
-    </r>
-  </si>
-  <si>
     <r>
       <t>Journals:</t>
     </r>
@@ -205,6 +173,18 @@
     </r>
   </si>
   <si>
+    <t>First author(s)</t>
+  </si>
+  <si>
+    <t>Will you use AI in this project? If yes, how so?</t>
+  </si>
+  <si>
+    <t>How will you account for attrition (i.e., competing risk of death)?</t>
+  </si>
+  <si>
+    <t>Modeling strengths (e.g. justification for choosing this model)</t>
+  </si>
+  <si>
     <r>
       <t>Resources (optional):</t>
     </r>
@@ -215,14 +195,37 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve"> Consider inlcuding links to papers that were influential in your thinking </t>
+      <t xml:space="preserve"> Consider including links to papers that were influential in your thinking </t>
     </r>
   </si>
   <si>
-    <t>First author(s)</t>
+    <r>
+      <t xml:space="preserve">Implementation steps: Copy this analysis plan to your preferred environment. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Fill out the initial analysis plan based on your project. Update the analysis plan as decisions are made; that is, whenever you make updates to the analysis or change coding choices, you should have this document open to record changes to the planned analysis. Remember this plan is to help promote reproducible research and will eventually be posted online. This document is for you, so modify it however you see fit!</t>
+    </r>
   </si>
   <si>
-    <t>Will you use AI in this project? If yes, how so?</t>
+    <t>What is the motivation for this work (~3 sentences)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brief summary of the data (cross sectional; longitudinal). Any oversamples or specific benefits of this data source? Study period: did you subsets data being used? </t>
+  </si>
+  <si>
+    <t>Eligibility criteria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any exclusions from the eligible to the analytic sample? </t>
+  </si>
+  <si>
+    <t>Number of people in the analytic sample and number of observations (if repeated outcome measures)</t>
   </si>
 </sst>
 </file>
@@ -308,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -338,9 +341,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -576,20 +576,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AB990"/>
+  <dimension ref="A1:AB991"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="16" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="50.1640625" style="15" customWidth="1"/>
-    <col min="2" max="2" width="37.6640625" style="12" customWidth="1"/>
-    <col min="3" max="3" width="2.6640625" style="12" customWidth="1"/>
-    <col min="4" max="6" width="37.6640625" style="12" customWidth="1"/>
-    <col min="7" max="7" width="2.6640625" style="12" customWidth="1"/>
-    <col min="8" max="8" width="37.6640625" style="12" customWidth="1"/>
-    <col min="9" max="9" width="2.6640625" style="12" customWidth="1"/>
-    <col min="10" max="10" width="37.6640625" style="12" customWidth="1"/>
-    <col min="11" max="11" width="2.6640625" style="12" customWidth="1"/>
-    <col min="12" max="12" width="37.6640625" style="12" customWidth="1"/>
-    <col min="13" max="16384" width="12.6640625" style="12"/>
+    <col min="1" max="1" width="50.1640625" style="14" customWidth="1"/>
+    <col min="2" max="2" width="37.6640625" style="11" customWidth="1"/>
+    <col min="3" max="3" width="2.6640625" style="11" customWidth="1"/>
+    <col min="4" max="6" width="37.6640625" style="11" customWidth="1"/>
+    <col min="7" max="7" width="2.6640625" style="11" customWidth="1"/>
+    <col min="8" max="8" width="37.6640625" style="11" customWidth="1"/>
+    <col min="9" max="9" width="2.6640625" style="11" customWidth="1"/>
+    <col min="10" max="10" width="37.6640625" style="11" customWidth="1"/>
+    <col min="11" max="11" width="2.6640625" style="11" customWidth="1"/>
+    <col min="12" max="12" width="37.6640625" style="11" customWidth="1"/>
+    <col min="13" max="16384" width="12.6640625" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="34" x14ac:dyDescent="0.15">
@@ -611,15 +611,15 @@
       </c>
       <c r="G1" s="2"/>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="I1" s="2"/>
       <c r="J1" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="K1" s="2"/>
       <c r="L1" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="M1" s="3"/>
       <c r="N1" s="3"/>
@@ -766,7 +766,7 @@
     </row>
     <row r="6" spans="1:28" ht="17" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="5"/>
@@ -798,7 +798,7 @@
     </row>
     <row r="7" spans="1:28" ht="17" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="5"/>
@@ -1084,7 +1084,7 @@
     </row>
     <row r="16" spans="1:28" ht="17" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="5"/>
@@ -1116,7 +1116,7 @@
     </row>
     <row r="17" spans="1:28" ht="68" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="5"/>
@@ -1178,7 +1178,7 @@
     </row>
     <row r="19" spans="1:28" ht="17" x14ac:dyDescent="0.15">
       <c r="A19" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B19" s="9"/>
       <c r="C19" s="10"/>
@@ -1210,7 +1210,7 @@
     </row>
     <row r="20" spans="1:28" ht="17" x14ac:dyDescent="0.15">
       <c r="A20" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="5"/>
@@ -1242,7 +1242,7 @@
     </row>
     <row r="21" spans="1:28" ht="34" x14ac:dyDescent="0.15">
       <c r="A21" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="5"/>
@@ -1274,7 +1274,7 @@
     </row>
     <row r="22" spans="1:28" ht="51" x14ac:dyDescent="0.15">
       <c r="A22" s="3" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="B22" s="3"/>
       <c r="C22" s="5"/>
@@ -1306,7 +1306,7 @@
     </row>
     <row r="23" spans="1:28" ht="17" x14ac:dyDescent="0.15">
       <c r="A23" s="3" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="5"/>
@@ -1338,7 +1338,7 @@
     </row>
     <row r="24" spans="1:28" ht="17" x14ac:dyDescent="0.15">
       <c r="A24" s="3" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="5"/>
@@ -1370,7 +1370,7 @@
     </row>
     <row r="25" spans="1:28" ht="34" x14ac:dyDescent="0.15">
       <c r="A25" s="3" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="5"/>
@@ -1402,7 +1402,7 @@
     </row>
     <row r="26" spans="1:28" ht="34" x14ac:dyDescent="0.15">
       <c r="A26" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="5"/>
@@ -1464,7 +1464,7 @@
     </row>
     <row r="28" spans="1:28" ht="51" x14ac:dyDescent="0.15">
       <c r="A28" s="9" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B28" s="9"/>
       <c r="C28" s="10"/>
@@ -1496,7 +1496,7 @@
     </row>
     <row r="29" spans="1:28" ht="68" x14ac:dyDescent="0.15">
       <c r="A29" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="5"/>
@@ -1528,7 +1528,7 @@
     </row>
     <row r="30" spans="1:28" ht="85" x14ac:dyDescent="0.15">
       <c r="A30" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="5"/>
@@ -1560,7 +1560,7 @@
     </row>
     <row r="31" spans="1:28" ht="68" x14ac:dyDescent="0.15">
       <c r="A31" s="3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="5"/>
@@ -1592,7 +1592,7 @@
     </row>
     <row r="32" spans="1:28" ht="68" x14ac:dyDescent="0.15">
       <c r="A32" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="5"/>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="33" spans="1:28" ht="85" x14ac:dyDescent="0.15">
       <c r="A33" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B33" s="3"/>
       <c r="C33" s="5"/>
@@ -1656,7 +1656,7 @@
     </row>
     <row r="34" spans="1:28" ht="34" x14ac:dyDescent="0.15">
       <c r="A34" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B34" s="3"/>
       <c r="C34" s="5"/>
@@ -1686,8 +1686,10 @@
       <c r="AA34" s="3"/>
       <c r="AB34" s="3"/>
     </row>
-    <row r="35" spans="1:28" x14ac:dyDescent="0.15">
-      <c r="A35" s="3"/>
+    <row r="35" spans="1:28" ht="34" x14ac:dyDescent="0.15">
+      <c r="A35" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="B35" s="3"/>
       <c r="C35" s="5"/>
       <c r="D35" s="3"/>
@@ -1716,75 +1718,73 @@
       <c r="AA35" s="3"/>
       <c r="AB35" s="3"/>
     </row>
-    <row r="36" spans="1:28" ht="17" x14ac:dyDescent="0.15">
-      <c r="A36" s="8" t="s">
-        <v>28</v>
+    <row r="36" spans="1:28" x14ac:dyDescent="0.15">
+      <c r="A36" s="3"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="5"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="5"/>
+      <c r="J36" s="3"/>
+      <c r="K36" s="5"/>
+      <c r="L36" s="3"/>
+      <c r="M36" s="3"/>
+      <c r="N36" s="3"/>
+      <c r="O36" s="3"/>
+      <c r="P36" s="3"/>
+      <c r="Q36" s="3"/>
+      <c r="R36" s="3"/>
+      <c r="S36" s="3"/>
+      <c r="T36" s="3"/>
+      <c r="U36" s="3"/>
+      <c r="V36" s="3"/>
+      <c r="W36" s="3"/>
+      <c r="X36" s="3"/>
+      <c r="Y36" s="3"/>
+      <c r="Z36" s="3"/>
+      <c r="AA36" s="3"/>
+      <c r="AB36" s="3"/>
+    </row>
+    <row r="37" spans="1:28" ht="17" x14ac:dyDescent="0.15">
+      <c r="A37" s="8" t="s">
+        <v>24</v>
       </c>
-      <c r="B36" s="9"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="9"/>
-      <c r="I36" s="10"/>
-      <c r="J36" s="9"/>
-      <c r="K36" s="10"/>
-      <c r="L36" s="9"/>
-      <c r="M36" s="9"/>
-      <c r="N36" s="9"/>
-      <c r="O36" s="9"/>
-      <c r="P36" s="9"/>
-      <c r="Q36" s="9"/>
-      <c r="R36" s="9"/>
-      <c r="S36" s="9"/>
-      <c r="T36" s="9"/>
-      <c r="U36" s="9"/>
-      <c r="V36" s="9"/>
-      <c r="W36" s="9"/>
-      <c r="X36" s="9"/>
-      <c r="Y36" s="9"/>
-      <c r="Z36" s="9"/>
-      <c r="AA36" s="9"/>
-      <c r="AB36" s="9"/>
-    </row>
-    <row r="37" spans="1:28" ht="51" x14ac:dyDescent="0.15">
-      <c r="A37" s="3" t="s">
-        <v>29</v>
+      <c r="B37" s="9"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="9"/>
+      <c r="I37" s="10"/>
+      <c r="J37" s="9"/>
+      <c r="K37" s="10"/>
+      <c r="L37" s="9"/>
+      <c r="M37" s="9"/>
+      <c r="N37" s="9"/>
+      <c r="O37" s="9"/>
+      <c r="P37" s="9"/>
+      <c r="Q37" s="9"/>
+      <c r="R37" s="9"/>
+      <c r="S37" s="9"/>
+      <c r="T37" s="9"/>
+      <c r="U37" s="9"/>
+      <c r="V37" s="9"/>
+      <c r="W37" s="9"/>
+      <c r="X37" s="9"/>
+      <c r="Y37" s="9"/>
+      <c r="Z37" s="9"/>
+      <c r="AA37" s="9"/>
+      <c r="AB37" s="9"/>
+    </row>
+    <row r="38" spans="1:28" ht="51" x14ac:dyDescent="0.15">
+      <c r="A38" s="3" t="s">
+        <v>25</v>
       </c>
-      <c r="B37" s="13"/>
-      <c r="C37" s="5"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="5"/>
-      <c r="H37" s="3"/>
-      <c r="I37" s="5"/>
-      <c r="J37" s="3"/>
-      <c r="K37" s="5"/>
-      <c r="L37" s="3"/>
-      <c r="M37" s="3"/>
-      <c r="N37" s="3"/>
-      <c r="O37" s="3"/>
-      <c r="P37" s="3"/>
-      <c r="Q37" s="3"/>
-      <c r="R37" s="3"/>
-      <c r="S37" s="3"/>
-      <c r="T37" s="3"/>
-      <c r="U37" s="3"/>
-      <c r="V37" s="3"/>
-      <c r="W37" s="3"/>
-      <c r="X37" s="3"/>
-      <c r="Y37" s="3"/>
-      <c r="Z37" s="3"/>
-      <c r="AA37" s="3"/>
-      <c r="AB37" s="3"/>
-    </row>
-    <row r="38" spans="1:28" ht="17" x14ac:dyDescent="0.15">
-      <c r="A38" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B38" s="3"/>
+      <c r="B38" s="12"/>
       <c r="C38" s="5"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
@@ -1812,9 +1812,9 @@
       <c r="AA38" s="3"/>
       <c r="AB38" s="3"/>
     </row>
-    <row r="39" spans="1:28" ht="34" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:28" ht="17" x14ac:dyDescent="0.15">
       <c r="A39" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B39" s="3"/>
       <c r="C39" s="5"/>
@@ -1846,7 +1846,7 @@
     </row>
     <row r="40" spans="1:28" ht="34" x14ac:dyDescent="0.15">
       <c r="A40" s="3" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="B40" s="3"/>
       <c r="C40" s="5"/>
@@ -1878,7 +1878,7 @@
     </row>
     <row r="41" spans="1:28" ht="34" x14ac:dyDescent="0.15">
       <c r="A41" s="3" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B41" s="3"/>
       <c r="C41" s="5"/>
@@ -1908,9 +1908,9 @@
       <c r="AA41" s="3"/>
       <c r="AB41" s="3"/>
     </row>
-    <row r="42" spans="1:28" ht="17" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:28" ht="34" x14ac:dyDescent="0.15">
       <c r="A42" s="3" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B42" s="3"/>
       <c r="C42" s="5"/>
@@ -1942,9 +1942,9 @@
     </row>
     <row r="43" spans="1:28" ht="17" x14ac:dyDescent="0.15">
       <c r="A43" s="3" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
-      <c r="B43" s="5"/>
+      <c r="B43" s="3"/>
       <c r="C43" s="5"/>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
@@ -1972,11 +1972,11 @@
       <c r="AA43" s="3"/>
       <c r="AB43" s="3"/>
     </row>
-    <row r="44" spans="1:28" x14ac:dyDescent="0.15">
-      <c r="A44" s="14" t="s">
-        <v>48</v>
+    <row r="44" spans="1:28" ht="17" x14ac:dyDescent="0.15">
+      <c r="A44" s="3" t="s">
+        <v>30</v>
       </c>
-      <c r="B44" s="11"/>
+      <c r="B44" s="5"/>
       <c r="C44" s="5"/>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
@@ -2005,75 +2005,75 @@
       <c r="AB44" s="3"/>
     </row>
     <row r="45" spans="1:28" x14ac:dyDescent="0.15">
-      <c r="C45" s="16"/>
-    </row>
-    <row r="46" spans="1:28" ht="34" x14ac:dyDescent="0.15">
-      <c r="A46" s="8" t="s">
-        <v>45</v>
+      <c r="A45" s="13" t="s">
+        <v>40</v>
       </c>
-      <c r="B46" s="9"/>
-      <c r="C46" s="10"/>
-      <c r="D46" s="9"/>
-      <c r="E46" s="9"/>
-      <c r="F46" s="9"/>
-      <c r="G46" s="10"/>
-      <c r="H46" s="9"/>
-      <c r="I46" s="10"/>
-      <c r="J46" s="9"/>
-      <c r="K46" s="10"/>
-      <c r="L46" s="9"/>
-      <c r="M46" s="9"/>
-      <c r="N46" s="9"/>
-      <c r="O46" s="9"/>
-      <c r="P46" s="9"/>
-      <c r="Q46" s="9"/>
-      <c r="R46" s="9"/>
-      <c r="S46" s="9"/>
-      <c r="T46" s="9"/>
-      <c r="U46" s="9"/>
-      <c r="V46" s="9"/>
-      <c r="W46" s="9"/>
-      <c r="X46" s="9"/>
-      <c r="Y46" s="9"/>
-      <c r="Z46" s="9"/>
-      <c r="AA46" s="9"/>
-      <c r="AB46" s="9"/>
-    </row>
-    <row r="47" spans="1:28" ht="17" x14ac:dyDescent="0.15">
-      <c r="A47" s="3" t="s">
-        <v>36</v>
+      <c r="B45" s="3"/>
+      <c r="C45" s="5"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="5"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="5"/>
+      <c r="L45" s="3"/>
+      <c r="M45" s="3"/>
+      <c r="N45" s="3"/>
+      <c r="O45" s="3"/>
+      <c r="P45" s="3"/>
+      <c r="Q45" s="3"/>
+      <c r="R45" s="3"/>
+      <c r="S45" s="3"/>
+      <c r="T45" s="3"/>
+      <c r="U45" s="3"/>
+      <c r="V45" s="3"/>
+      <c r="W45" s="3"/>
+      <c r="X45" s="3"/>
+      <c r="Y45" s="3"/>
+      <c r="Z45" s="3"/>
+      <c r="AA45" s="3"/>
+      <c r="AB45" s="3"/>
+    </row>
+    <row r="46" spans="1:28" x14ac:dyDescent="0.15">
+      <c r="C46" s="15"/>
+    </row>
+    <row r="47" spans="1:28" ht="34" x14ac:dyDescent="0.15">
+      <c r="A47" s="8" t="s">
+        <v>38</v>
       </c>
-      <c r="B47" s="3"/>
-      <c r="C47" s="5"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="5"/>
-      <c r="H47" s="3"/>
-      <c r="I47" s="5"/>
-      <c r="J47" s="3"/>
-      <c r="K47" s="5"/>
-      <c r="L47" s="3"/>
-      <c r="M47" s="3"/>
-      <c r="N47" s="3"/>
-      <c r="O47" s="3"/>
-      <c r="P47" s="3"/>
-      <c r="Q47" s="3"/>
-      <c r="R47" s="3"/>
-      <c r="S47" s="3"/>
-      <c r="T47" s="3"/>
-      <c r="U47" s="3"/>
-      <c r="V47" s="3"/>
-      <c r="W47" s="3"/>
-      <c r="X47" s="3"/>
-      <c r="Y47" s="3"/>
-      <c r="Z47" s="3"/>
-      <c r="AA47" s="3"/>
-      <c r="AB47" s="3"/>
-    </row>
-    <row r="48" spans="1:28" ht="34" x14ac:dyDescent="0.15">
+      <c r="B47" s="9"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="9"/>
+      <c r="I47" s="10"/>
+      <c r="J47" s="9"/>
+      <c r="K47" s="10"/>
+      <c r="L47" s="9"/>
+      <c r="M47" s="9"/>
+      <c r="N47" s="9"/>
+      <c r="O47" s="9"/>
+      <c r="P47" s="9"/>
+      <c r="Q47" s="9"/>
+      <c r="R47" s="9"/>
+      <c r="S47" s="9"/>
+      <c r="T47" s="9"/>
+      <c r="U47" s="9"/>
+      <c r="V47" s="9"/>
+      <c r="W47" s="9"/>
+      <c r="X47" s="9"/>
+      <c r="Y47" s="9"/>
+      <c r="Z47" s="9"/>
+      <c r="AA47" s="9"/>
+      <c r="AB47" s="9"/>
+    </row>
+    <row r="48" spans="1:28" ht="17" x14ac:dyDescent="0.15">
       <c r="A48" s="3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B48" s="3"/>
       <c r="C48" s="5"/>
@@ -2103,8 +2103,10 @@
       <c r="AA48" s="3"/>
       <c r="AB48" s="3"/>
     </row>
-    <row r="49" spans="1:28" x14ac:dyDescent="0.15">
-      <c r="A49" s="3"/>
+    <row r="49" spans="1:28" ht="34" x14ac:dyDescent="0.15">
+      <c r="A49" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="B49" s="3"/>
       <c r="C49" s="5"/>
       <c r="D49" s="3"/>
@@ -2133,72 +2135,72 @@
       <c r="AA49" s="3"/>
       <c r="AB49" s="3"/>
     </row>
-    <row r="50" spans="1:28" ht="34" x14ac:dyDescent="0.15">
-      <c r="A50" s="8" t="s">
-        <v>46</v>
+    <row r="50" spans="1:28" x14ac:dyDescent="0.15">
+      <c r="A50" s="3"/>
+      <c r="B50" s="3"/>
+      <c r="C50" s="5"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="5"/>
+      <c r="J50" s="3"/>
+      <c r="K50" s="5"/>
+      <c r="L50" s="3"/>
+      <c r="M50" s="3"/>
+      <c r="N50" s="3"/>
+      <c r="O50" s="3"/>
+      <c r="P50" s="3"/>
+      <c r="Q50" s="3"/>
+      <c r="R50" s="3"/>
+      <c r="S50" s="3"/>
+      <c r="T50" s="3"/>
+      <c r="U50" s="3"/>
+      <c r="V50" s="3"/>
+      <c r="W50" s="3"/>
+      <c r="X50" s="3"/>
+      <c r="Y50" s="3"/>
+      <c r="Z50" s="3"/>
+      <c r="AA50" s="3"/>
+      <c r="AB50" s="3"/>
+    </row>
+    <row r="51" spans="1:28" ht="34" x14ac:dyDescent="0.15">
+      <c r="A51" s="8" t="s">
+        <v>43</v>
       </c>
-      <c r="B50" s="9"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="9"/>
-      <c r="F50" s="9"/>
-      <c r="G50" s="10"/>
-      <c r="H50" s="9"/>
-      <c r="I50" s="10"/>
-      <c r="J50" s="9"/>
-      <c r="K50" s="10"/>
-      <c r="L50" s="9"/>
-      <c r="M50" s="9"/>
-      <c r="N50" s="9"/>
-      <c r="O50" s="9"/>
-      <c r="P50" s="9"/>
-      <c r="Q50" s="9"/>
-      <c r="R50" s="9"/>
-      <c r="S50" s="9"/>
-      <c r="T50" s="9"/>
-      <c r="U50" s="9"/>
-      <c r="V50" s="9"/>
-      <c r="W50" s="9"/>
-      <c r="X50" s="9"/>
-      <c r="Y50" s="9"/>
-      <c r="Z50" s="9"/>
-      <c r="AA50" s="9"/>
-      <c r="AB50" s="9"/>
-    </row>
-    <row r="51" spans="1:28" ht="17" x14ac:dyDescent="0.15">
-      <c r="A51" s="3" t="s">
-        <v>38</v>
+      <c r="B51" s="9"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="9"/>
+      <c r="F51" s="9"/>
+      <c r="G51" s="10"/>
+      <c r="H51" s="9"/>
+      <c r="I51" s="10"/>
+      <c r="J51" s="9"/>
+      <c r="K51" s="10"/>
+      <c r="L51" s="9"/>
+      <c r="M51" s="9"/>
+      <c r="N51" s="9"/>
+      <c r="O51" s="9"/>
+      <c r="P51" s="9"/>
+      <c r="Q51" s="9"/>
+      <c r="R51" s="9"/>
+      <c r="S51" s="9"/>
+      <c r="T51" s="9"/>
+      <c r="U51" s="9"/>
+      <c r="V51" s="9"/>
+      <c r="W51" s="9"/>
+      <c r="X51" s="9"/>
+      <c r="Y51" s="9"/>
+      <c r="Z51" s="9"/>
+      <c r="AA51" s="9"/>
+      <c r="AB51" s="9"/>
+    </row>
+    <row r="52" spans="1:28" ht="17" x14ac:dyDescent="0.15">
+      <c r="A52" s="3" t="s">
+        <v>33</v>
       </c>
-      <c r="B51" s="3"/>
-      <c r="C51" s="5"/>
-      <c r="D51" s="3"/>
-      <c r="E51" s="3"/>
-      <c r="F51" s="3"/>
-      <c r="G51" s="5"/>
-      <c r="H51" s="3"/>
-      <c r="I51" s="5"/>
-      <c r="J51" s="3"/>
-      <c r="K51" s="5"/>
-      <c r="L51" s="3"/>
-      <c r="M51" s="3"/>
-      <c r="N51" s="3"/>
-      <c r="O51" s="3"/>
-      <c r="P51" s="3"/>
-      <c r="Q51" s="3"/>
-      <c r="R51" s="3"/>
-      <c r="S51" s="3"/>
-      <c r="T51" s="3"/>
-      <c r="U51" s="3"/>
-      <c r="V51" s="3"/>
-      <c r="W51" s="3"/>
-      <c r="X51" s="3"/>
-      <c r="Y51" s="3"/>
-      <c r="Z51" s="3"/>
-      <c r="AA51" s="3"/>
-      <c r="AB51" s="3"/>
-    </row>
-    <row r="52" spans="1:28" x14ac:dyDescent="0.15">
-      <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="5"/>
       <c r="D52" s="3"/>
@@ -30367,6 +30369,36 @@
       <c r="AA990" s="3"/>
       <c r="AB990" s="3"/>
     </row>
+    <row r="991" spans="1:28" x14ac:dyDescent="0.15">
+      <c r="A991" s="3"/>
+      <c r="B991" s="3"/>
+      <c r="C991" s="5"/>
+      <c r="D991" s="3"/>
+      <c r="E991" s="3"/>
+      <c r="F991" s="3"/>
+      <c r="G991" s="5"/>
+      <c r="H991" s="3"/>
+      <c r="I991" s="5"/>
+      <c r="J991" s="3"/>
+      <c r="K991" s="5"/>
+      <c r="L991" s="3"/>
+      <c r="M991" s="3"/>
+      <c r="N991" s="3"/>
+      <c r="O991" s="3"/>
+      <c r="P991" s="3"/>
+      <c r="Q991" s="3"/>
+      <c r="R991" s="3"/>
+      <c r="S991" s="3"/>
+      <c r="T991" s="3"/>
+      <c r="U991" s="3"/>
+      <c r="V991" s="3"/>
+      <c r="W991" s="3"/>
+      <c r="X991" s="3"/>
+      <c r="Y991" s="3"/>
+      <c r="Z991" s="3"/>
+      <c r="AA991" s="3"/>
+      <c r="AB991" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>